<commit_message>
Fincalidad para conexión remota de Ngrok
</commit_message>
<xml_diff>
--- a/public/Docs/NWI043_Brief.xlsx
+++ b/public/Docs/NWI043_Brief.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TRABAJO\Newrona\Projects\IA\LM Studio\TypeScript\ts_v2_Vite\public\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC92C9DB-097E-45D7-B1E3-5FEFB26DC749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76051937-97AD-4336-BDBF-6141D6B27A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base de conocimiento" sheetId="2" r:id="rId1"/>
@@ -40,10 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="140">
-  <si>
-    <t>Tema</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="134">
   <si>
     <t>Pregunta</t>
   </si>
@@ -52,9 +49,6 @@
   </si>
   <si>
     <t>Texto final</t>
-  </si>
-  <si>
-    <t>Newrona</t>
   </si>
   <si>
     <t>¿Qué es Newrona?</t>
@@ -172,9 +166,6 @@
 Nuestro horario de atención es de lunes a viernes, de 8:00 a.m. a 5:00 p.m.</t>
   </si>
   <si>
-    <t>Core de Negocio</t>
-  </si>
-  <si>
     <t>¿Con qué sectores trabaja Newrona?</t>
   </si>
   <si>
@@ -318,9 +309,6 @@
   </si>
   <si>
     <t>El tiempo de desarrollo para un proyecto con Realidad Aumentada puede variar bastante. En general, podría tomarnos unas 4 semanas o más. Sin embargo, cada proyecto es único y tiene sus propios desafíos y objetivos, por lo que la duración puede cambiar.</t>
-  </si>
-  <si>
-    <t>Tecnologías Inmersivas</t>
   </si>
   <si>
     <t>¿Qué son las tecnologías inmersivas?</t>
@@ -548,9 +536,6 @@
 - A través de escenarios interactivos, como avatares holográficos.</t>
   </si>
   <si>
-    <t>Uso de las Tecnologías en el sector Industrial</t>
-  </si>
-  <si>
     <t>¿Qué es un entrenamiento inmersivo?</t>
   </si>
   <si>
@@ -607,9 +592,6 @@
 - Optimización de procesos, visualizando y ajustando flujos de trabajo antes de implementarlos.
 -Reducción de costos asociados a errores humanos o paros de producción.
 - Mejora del diseño de plantas y maquinaria mediante modelos 3D interactivos.</t>
-  </si>
-  <si>
-    <t>Personalidad</t>
   </si>
   <si>
     <t>¿Quien eres?</t>
@@ -1137,7 +1119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1161,7 +1143,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1236,7 +1217,6 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1268,39 +1248,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1518,17 +1465,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8A82E72-D491-4521-966E-A15DEA9E51CF}">
-  <dimension ref="A1:E56"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D56"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" style="12" customWidth="1"/>
-    <col min="3" max="3" width="58.85546875" style="12" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="94.140625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="72.28515625" customWidth="1"/>
+    <col min="1" max="1" width="37.7109375" style="11" customWidth="1"/>
+    <col min="2" max="2" width="58.85546875" style="11" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="94.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="72.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1538,600 +1484,530 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="51" t="s">
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="B3" s="14" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="51"/>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="15" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="B4" s="15" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="51"/>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="16" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="B5" s="16" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="63" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="51"/>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="17" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="B6" s="17" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="51"/>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="18" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="B7" s="18" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="51"/>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="19" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="B8" s="19" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="51"/>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="20" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="B9" s="20" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="51"/>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="21" t="s">
+    </row>
+    <row r="10" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="B10" s="18" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="51"/>
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="19" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="B11" s="18" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="51"/>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="19" t="s">
+    </row>
+    <row r="12" spans="1:3" s="29" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="10"/>
+    </row>
+    <row r="13" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="B13" s="22" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" s="30" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="9"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="11"/>
-    </row>
-    <row r="13" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="53" t="s">
+      <c r="C13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="13" t="s">
+    </row>
+    <row r="14" spans="1:3" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="B14" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="54"/>
-      <c r="B14" s="6" t="s">
+    <row r="15" spans="1:3" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="B15" s="24"/>
+      <c r="C15" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="4" t="s">
+    </row>
+    <row r="16" spans="1:3" ht="138" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="54"/>
-      <c r="B15" s="7" t="s">
+      <c r="B16" s="22"/>
+      <c r="C16" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="25"/>
-      <c r="D15" s="38" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="138" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="54"/>
-      <c r="B16" s="7" t="s">
+      <c r="B17" s="22"/>
+      <c r="C17" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="38" t="s">
+      <c r="D17" s="35"/>
+    </row>
+    <row r="18" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="54"/>
-      <c r="B17" s="7" t="s">
+      <c r="B18" s="22"/>
+      <c r="C18" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="38" t="s">
+    </row>
+    <row r="19" spans="1:4" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="37"/>
-    </row>
-    <row r="18" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="54"/>
-      <c r="B18" s="7" t="s">
+      <c r="B19" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="38" t="s">
+      <c r="C19" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="54"/>
-      <c r="B19" s="6" t="s">
+    <row r="20" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="54"/>
-      <c r="B20" s="6" t="s">
+    <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="26" t="s">
+      <c r="B21" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="54"/>
-      <c r="B21" s="6" t="s">
+    <row r="22" spans="1:4" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="B22" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="55"/>
-      <c r="B22" s="6" t="s">
+    <row r="23" spans="1:4" s="29" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="9"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="30"/>
+    </row>
+    <row r="24" spans="1:4" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="B24" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="C24" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="30" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="31"/>
-    </row>
-    <row r="24" spans="1:5" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="56" t="s">
+    <row r="25" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B25" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C25" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D24" s="4" t="s">
+    </row>
+    <row r="26" spans="1:4" ht="48" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="54" x14ac:dyDescent="0.2">
-      <c r="A25" s="57"/>
-      <c r="B25" s="6" t="s">
+      <c r="B26" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C26" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D25" s="4" t="s">
+    </row>
+    <row r="27" spans="1:4" ht="153" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="67.5" x14ac:dyDescent="0.2">
-      <c r="A26" s="57"/>
-      <c r="B26" s="6" t="s">
+      <c r="B27" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C27" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D26" s="4" t="s">
+    </row>
+    <row r="28" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="153" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="57"/>
-      <c r="B27" s="6" t="s">
+      <c r="B28" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C28" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="4" t="s">
+    </row>
+    <row r="29" spans="1:4" ht="142.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="6" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="57"/>
-      <c r="B28" s="6" t="s">
+      <c r="B29" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C29" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="4" t="s">
+    </row>
+    <row r="30" spans="1:4" ht="73.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="142.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="57"/>
-      <c r="B29" s="6" t="s">
+      <c r="B30" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C30" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D29" s="4" t="s">
+    </row>
+    <row r="31" spans="1:4" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="6" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="73.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="57"/>
-      <c r="B30" s="6" t="s">
+      <c r="B31" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="C30" s="23" t="s">
+      <c r="C31" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D30" s="4" t="s">
+    </row>
+    <row r="32" spans="1:4" ht="96.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="57"/>
-      <c r="B31" s="6" t="s">
+      <c r="B32" s="22"/>
+      <c r="C32" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="23" t="s">
+    </row>
+    <row r="33" spans="1:3" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="B33" s="25" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" ht="96.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="57"/>
-      <c r="B32" s="6" t="s">
+      <c r="C33" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="4" t="s">
+    </row>
+    <row r="34" spans="1:3" ht="108.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="57"/>
-      <c r="B33" s="6" t="s">
+      <c r="B34" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C34" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="D33" s="4" t="s">
+    </row>
+    <row r="35" spans="1:3" ht="120" x14ac:dyDescent="0.2">
+      <c r="A35" s="6" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="108.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="57"/>
-      <c r="B34" s="6" t="s">
+      <c r="B35" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="C34" s="23" t="s">
+      <c r="C35" s="34" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D34" s="29" t="s">
+      <c r="B36" s="22" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="135" x14ac:dyDescent="0.2">
-      <c r="A35" s="57"/>
-      <c r="B35" s="6" t="s">
+      <c r="C36" s="33" t="s">
         <v>95</v>
       </c>
-      <c r="C35" s="26" t="s">
+    </row>
+    <row r="37" spans="1:3" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="D35" s="35" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="57"/>
-      <c r="B36" s="6" t="s">
+      <c r="B37" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C36" s="23" t="s">
+      <c r="C37" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D36" s="34" t="s">
+    </row>
+    <row r="38" spans="1:3" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="57"/>
-      <c r="B37" s="6" t="s">
+      <c r="B38" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C38" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D37" s="4" t="s">
+    </row>
+    <row r="39" spans="1:3" ht="93.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="6" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="57"/>
-      <c r="B38" s="6" t="s">
+      <c r="B39" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="C38" s="19" t="s">
+      <c r="C39" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D38" s="4" t="s">
+    </row>
+    <row r="40" spans="1:3" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="93.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="57"/>
-      <c r="B39" s="6" t="s">
+      <c r="B40" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="C39" s="19" t="s">
+      <c r="C40" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D39" s="4" t="s">
+    </row>
+    <row r="41" spans="1:3" s="29" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="10"/>
+      <c r="B41" s="27"/>
+      <c r="C41" s="30"/>
+    </row>
+    <row r="42" spans="1:3" ht="69" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="58"/>
-      <c r="B40" s="6" t="s">
+      <c r="B42" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="C40" s="23" t="s">
+      <c r="C42" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="D40" s="4" t="s">
+    </row>
+    <row r="43" spans="1:3" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="6" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" s="30" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="9"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="31"/>
-    </row>
-    <row r="42" spans="1:4" ht="69" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="52" t="s">
+      <c r="B43" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="C43" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C42" s="26" t="s">
+    </row>
+    <row r="44" spans="1:3" ht="102" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="B44" s="22" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="52"/>
-      <c r="B43" s="6" t="s">
+      <c r="C44" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C43" s="26" t="s">
+    </row>
+    <row r="45" spans="1:3" ht="134.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="B45" s="22" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" ht="102" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="52"/>
-      <c r="B44" s="6" t="s">
+      <c r="C45" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="C44" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="134.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="52"/>
-      <c r="B45" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C45" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="36"/>
+    </row>
+    <row r="46" spans="1:3" s="29" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="30"/>
       <c r="B46" s="31"/>
       <c r="C46" s="32"/>
-      <c r="D46" s="33"/>
-    </row>
-    <row r="47" spans="1:4" ht="365.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="48" t="s">
+    </row>
+    <row r="47" spans="1:3" ht="365.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="44"/>
+      <c r="C47" s="36" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="42" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" s="37"/>
+      <c r="C48" s="36" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="45" t="s">
+        <v>124</v>
+      </c>
+      <c r="B49" s="37"/>
+      <c r="C49" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="B47" s="45" t="s">
+    </row>
+    <row r="50" spans="1:3" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="45"/>
+      <c r="B50" s="37"/>
+      <c r="C50" s="39" t="s">
         <v>126</v>
       </c>
-      <c r="C47" s="46"/>
-      <c r="D47" s="38" t="s">
+    </row>
+    <row r="51" spans="1:3" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="45"/>
+      <c r="B51" s="40"/>
+      <c r="C51" s="41" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="49"/>
-      <c r="B48" s="44" t="s">
+    <row r="52" spans="1:3" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="45"/>
+      <c r="B52" s="40"/>
+      <c r="C52" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="C48" s="39"/>
-      <c r="D48" s="38" t="s">
+    </row>
+    <row r="53" spans="1:3" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="45"/>
+      <c r="B53" s="40"/>
+      <c r="C53" s="39" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="49"/>
-      <c r="B49" s="47" t="s">
-        <v>130</v>
-      </c>
-      <c r="C49" s="39"/>
-      <c r="D49" s="40" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="49"/>
-      <c r="B50" s="47"/>
-      <c r="C50" s="39"/>
-      <c r="D50" s="41" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="49"/>
-      <c r="B51" s="47"/>
-      <c r="C51" s="42"/>
-      <c r="D51" s="43" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="49"/>
-      <c r="B52" s="47"/>
-      <c r="C52" s="42"/>
-      <c r="D52" s="43" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="399.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="50"/>
-      <c r="B53" s="47"/>
-      <c r="C53" s="42"/>
-      <c r="D53" s="41" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C56" s="26"/>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B56" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="A47:A53"/>
-    <mergeCell ref="A2:A11"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="A13:A22"/>
-    <mergeCell ref="A24:A40"/>
+  <mergeCells count="1">
+    <mergeCell ref="A49:A53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2150,20 +2026,20 @@
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" ht="13.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="90.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C4" s="1"/>
     </row>
@@ -2182,6 +2058,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8d039caa-5e68-4b24-bb5f-f0b14b378ae7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e8539436-38c8-4b16-b514-92d303eb059d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101002CB8F03847968542941A8073265A74CB" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0c5ae6f0c9073defa7c13228c79764c9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8d039caa-5e68-4b24-bb5f-f0b14b378ae7" xmlns:ns3="e8539436-38c8-4b16-b514-92d303eb059d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="27eacf4a78c787487ec2cfc1b20d48b5" ns2:_="" ns3:_="">
     <xsd:import namespace="8d039caa-5e68-4b24-bb5f-f0b14b378ae7"/>
@@ -2388,17 +2275,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8d039caa-5e68-4b24-bb5f-f0b14b378ae7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e8539436-38c8-4b16-b514-92d303eb059d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{293F8DEE-ED4B-469E-AF52-5340F86FF98C}">
   <ds:schemaRefs>
@@ -2408,6 +2284,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A60E7A1E-BE31-41BB-988E-18B074B77898}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="8d039caa-5e68-4b24-bb5f-f0b14b378ae7"/>
+    <ds:schemaRef ds:uri="e8539436-38c8-4b16-b514-92d303eb059d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A2DB34D-08BF-4F66-A8C5-9F048C46CCB2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2426,17 +2313,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A60E7A1E-BE31-41BB-988E-18B074B77898}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="8d039caa-5e68-4b24-bb5f-f0b14b378ae7"/>
-    <ds:schemaRef ds:uri="e8539436-38c8-4b16-b514-92d303eb059d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e20b666e-bc5d-47f2-89f9-fcd7cbf4b9bf}" enabled="0" method="" siteId="{e20b666e-bc5d-47f2-89f9-fcd7cbf4b9bf}" removed="1"/>

</xml_diff>